<commit_message>
align formating for table
</commit_message>
<xml_diff>
--- a/SOA-C03/SOA-C03-ExamTopics-Questions.xlsx
+++ b/SOA-C03/SOA-C03-ExamTopics-Questions.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://jetstarairways-my.sharepoint.com/personal/balraj_singh_jetstar_com/Documents/Balraj_D_Laptop_Drive/DevOps_Master/Learn-AI-MCP_ML/SOA-C03/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="542" documentId="8_{6D7FEDCE-BF68-490E-8FEE-13CF0653E58D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0FE4361D-3581-4290-965D-AFE092E3CEC4}"/>
+  <xr:revisionPtr revIDLastSave="543" documentId="8_{6D7FEDCE-BF68-490E-8FEE-13CF0653E58D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BBADE943-6160-42DA-A907-998034BE66F4}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="-210" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{D730D107-BEC6-4E62-9FED-4CE422768F8C}"/>
   </bookViews>
@@ -587,7 +587,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -626,6 +626,14 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="4">
     <fill>
@@ -656,10 +664,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -682,12 +691,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="centerContinuous"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="1" applyAlignment="1">
       <alignment shrinkToFit="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="3">
@@ -2726,7 +2735,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>179</v>
       </c>
       <c r="B1" s="5" t="s">
@@ -3409,7 +3418,7 @@
       <c r="A77" s="1">
         <v>75</v>
       </c>
-      <c r="B77" s="8" t="s">
+      <c r="B77" t="s">
         <v>120</v>
       </c>
     </row>
@@ -4358,6 +4367,9 @@
   <conditionalFormatting sqref="B2:B1048576">
     <cfRule type="duplicateValues" dxfId="0" priority="5"/>
   </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink ref="A1" r:id="rId1" xr:uid="{E4BE23F5-8686-4318-92B6-7D7B715CDD5E}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>